<commit_message>
CV websites: Natalie's examples (Betz first) replace the web-search list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/cv.xlsx
+++ b/downloads/cv.xlsx
@@ -529,11 +529,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Practice websites that post a CV, and how (12)</t>
+          <t>Practice websites that post a CV, and how (10): Natalie's examples, Dr. Joe Betz first</t>
         </is>
       </c>
     </row>
@@ -7222,14 +7222,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="64" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7262,12 +7262,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Austrager, Howard, DC</t>
+          <t>Betz, Joseph W, DC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>metrowestspineclinic.com</t>
+          <t>modernchiropracticcenter.com</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -7282,19 +7282,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>'click HERE' for CV on About Us (PDF)</t>
+          <t>Bio page with a "Link to Curriculum Vitae" button that opens the full CV (PDF, September 2026). The set-up to copy.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bienenfeld, Joel, DC</t>
+          <t>Bisaccia, John and Marna, DC (NMR certified)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>drjoelchiropractic.com</t>
+          <t>willistonchiropractic.com</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -7309,19 +7309,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>'Dr. Joel's CV' page plus a downloadable PDF</t>
+          <t>About page with each doctor's bio and NMR certification; no CV.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Davis, Timothy, MD</t>
+          <t>Casazza, Lance, DC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sourcehealthcare.com</t>
+          <t>sacramentochiropractic.com</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -7336,24 +7336,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>'See Dr. Davis' Curriculum Vitae' button (MD, sports medicine)</t>
+          <t>Team page with a full bio for each doctor (education, experience, certifications, books); no separate CV.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Frisch, Todd, DC</t>
+          <t>Cool Chiropractic (Sacramento)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>shapereclaimed.com</t>
+          <t>coolchiropracticsac.com</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -7363,24 +7363,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CV PDF linked from About</t>
+          <t>Team page with a full bio for each doctor; no separate CV.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Griffith, Alexis, DC</t>
+          <t>Fish, Gene, DC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>impowersportsperformance.com</t>
+          <t>genesischiroclinic.com</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>open the page</t>
+          <t>open the CV</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -7390,24 +7390,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CV section written into the About page</t>
+          <t>About page with a "See Dr. Fish's CV" button (PDF).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jaime, Joe, DC</t>
+          <t>Horrigan, Joseph, DC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>onthegosportschiro.com</t>
+          <t>scuhs.edu</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -7417,19 +7417,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Curriculum Vitae page in the site menu</t>
+          <t>Faculty bio page; no CV.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Junnila, Rick, DC</t>
+          <t>Moreau, William (Bill), DC, DACBSP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>doc.vortala.com</t>
+          <t>neurosportspineandconcussion.com</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -7444,24 +7444,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>'Dr. Junnila's Curriculum Vitae' link (PDF, 2026)</t>
+          <t>Team page with a CV summary and drop-downs; a Curriculum Vitae page with highlights and a "Download Full Curriculum Vitae (PDF)" button; instructor and speaker bios elsewhere.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>McDowell, Gary, DC</t>
+          <t>P2 Sports Care</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>my.onlinechiro.com</t>
+          <t>p2sportscare.com</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -7471,24 +7471,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CV and accolades PDF on About Us</t>
+          <t>Team page with a full bio for each doctor; no separate CV.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Poller, Wayne, DC</t>
+          <t>Sorrentino, Anne, DC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>drpoller.com</t>
+          <t>drannesorrentino.com</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -7498,24 +7498,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>'Curriculum Vitae - CLICK HERE' (PDF on letterhead)</t>
+          <t>Short bio with credentials after the name; no CV.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Reinboldt, Daniel, DC</t>
+          <t>Young, Tom, DC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>greenvillespineandjoint.com</t>
+          <t>countryside-chiropractic.com</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -7525,61 +7525,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>'CLICK HERE' for CV (PDF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Thomas, William, DC</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>drtchiro.com</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>open the CV</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>'CV (Curriculum Vitae)' link on homepage</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Whalen, Wayne, DC</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>drwhalen.com</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>open the CV</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>'Curriculum Vitae' tab under Meet the Doctors</t>
+          <t>Short bio with credentials after the name; no CV.</t>
         </is>
       </c>
     </row>
@@ -7605,10 +7551,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7624,7 +7566,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -7660,12 +7602,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bart Green</t>
+          <t>Alexis Griffith</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>nuhs.edu</t>
+          <t>impowersportsperformance.com</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -7687,17 +7629,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Betz, Joseph W</t>
+          <t>Bart Green</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>modernchiropracticcenter.com</t>
+          <t>nuhs.edu</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -7707,7 +7649,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sports chiropractor</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
@@ -7741,17 +7683,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fish, Gene</t>
+          <t>Jamie Shortz</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>genesischiroclinic.com</t>
+          <t>pacificperformancechiro.com</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -7761,24 +7703,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sports chiropractor</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jamie Shortz</t>
+          <t>Joe Jaime</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pacificperformancechiro.com</t>
+          <t>onthegosportschiro.com</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>open the page</t>
+          <t>open the CV</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -7795,12 +7737,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Michael T. Fanning DC, DACBSP, RMSK, CSCS, *D</t>
+          <t>Joel Bienenfeld</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>scuhs.edu</t>
+          <t>drjoelchiropractic.com</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -7822,17 +7764,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moreau, William</t>
+          <t>Michael T. Fanning DC, DACBSP, RMSK, CSCS, *D</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>neurosportspineandconcussion.com</t>
+          <t>scuhs.edu</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -7842,7 +7784,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sports chiropractor</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
All CV lists on the Sample CVs page; directory keeps only people and websites
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/cv.xlsx
+++ b/downloads/cv.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="California CVs online" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Chiro Directory CVs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CVs from other searches" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Websites that post a CV" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Websites that post a CV" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="California CVs online" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Chiro Directory CVs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CVs from other searches" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sports and NMR chiro CVs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books by chiropractors" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
@@ -480,60 +480,60 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>California CVs online</t>
+          <t>Websites that post a CV</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>163</v>
+        <v>11</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>California chiropractor CVs found online (163)</t>
+          <t>Websites that post a CV, and how (11)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>US Chiro Directory CVs</t>
+          <t>California CVs online</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>68</v>
+        <v>163</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CV pages on US Chiro Directory (68)</t>
+          <t>California chiropractor CVs found online (163)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>CVs from other searches</t>
+          <t>US Chiro Directory CVs</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CVs and biographies from other web searches (40)</t>
+          <t>CV pages on US Chiro Directory (68)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Websites that post a CV</t>
+          <t>CVs from other searches</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Practice websites that post a CV, and how (10): Natalie's examples, Dr. Joe Betz first</t>
+          <t>CVs and biographies from other web searches (40)</t>
         </is>
       </c>
     </row>
@@ -544,11 +544,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CVs of sports, CCSP, NFL team and NMR chiropractors (10)</t>
+          <t>CVs of sports, CCSP, NFL team and NMR chiropractors (13)</t>
         </is>
       </c>
     </row>
@@ -581,6 +581,395 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="49" customWidth="1" min="1" max="1"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Doctor</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>About or team page</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Other pages</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>How the site shows it</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Betz, Joseph W, DC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Modern Chiropractic Center</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>modernchiropracticcenter.com</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bio page with a "Link to Curriculum Vitae" button that opens the full CV (PDF, September 2026). The set-up to copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Moreau, William (Bill), DC, DACBSP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NeuroSport Spine and Concussion</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>neurosportspineandconcussion.com</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>CV (PDF) · CV (PDF) · dconline.org · ncmic.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Team page with a CV summary and drop-downs; a Curriculum Vitae page with highlights and a "Download Full Curriculum Vitae (PDF)" button; instructor and speaker bios elsewhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fish, Gene, DC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Genesis Chiropractic</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>genesischiroclinic.com</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>About page with a "See Dr. Fish's CV" button (PDF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Injury and Spinecare Chiropractic, La Crescenta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Injury and Spinecare Chiropractic</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>injuryandspinecare.com</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>About page with "Click to view CV"; the CV is a page on US Chiro Directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Casazza, Lance, DC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sacramento Chiropractic</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>sacramentochiropractic.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>sacramentochiropractic.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Team page with a full bio for each doctor (education, experience, certifications, books); no separate CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cool Chiropractic (Sacramento)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cool Chiropractic</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>coolchiropracticsac.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Team page with a full bio for each doctor; no separate CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P2 Sports Care</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P2 Sports Care</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>p2sportscare.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Team page with a full bio for each doctor; no separate CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sorrentino, Anne, DC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dr. Anne Sorrentino</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>drannesorrentino.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Short bio with credentials after the name; no CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Young, Tom, DC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Countryside Chiropractic</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>countryside-chiropractic.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Short bio with credentials after the name; no CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Horrigan, Joseph, DC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Southern California University of Health Sciences</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>scuhs.edu</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Faculty bio page; no CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bisaccia, John and Marna, DC (NMR certified)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Williston Chiropractic &amp; Sportsmedicine</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>willistonchiropractic.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>no separate CV</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>About page with each doctor's bio and NMR certification; no CV.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId17"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4536,7 +4925,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6212,7 +6601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7216,20 +7605,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="47" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="72" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7255,24 +7644,24 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>How the site shows it</t>
+          <t>Group</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Betz, Joseph W, DC</t>
+          <t>Alexis Griffith</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>modernchiropracticcenter.com</t>
+          <t>impowersportsperformance.com</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>open the CV</t>
+          <t>open the page</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -7282,19 +7671,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bio page with a "Link to Curriculum Vitae" button that opens the full CV (PDF, September 2026). The set-up to copy.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bisaccia, John and Marna, DC (NMR certified)</t>
+          <t>Bart Green</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>willistonchiropractic.com</t>
+          <t>nuhs.edu</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -7309,24 +7698,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>About page with each doctor's bio and NMR certification; no CV.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Casazza, Lance, DC</t>
+          <t>Betz, Joseph W</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sacramentochiropractic.com</t>
+          <t>modernchiropracticcenter.com</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>open the page</t>
+          <t>open the CV</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -7336,19 +7725,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Team page with a full bio for each doctor (education, experience, certifications, books); no separate CV.</t>
+          <t>Sports chiropractor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cool Chiropractic (Sacramento)</t>
+          <t>Christian Brown</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>coolchiropracticsac.com</t>
+          <t>dhaj7-cepo.com</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -7363,14 +7752,14 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Team page with a full bio for each doctor; no separate CV.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fish, Gene, DC</t>
+          <t>Fish, Gene</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7390,19 +7779,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>About page with a "See Dr. Fish's CV" button (PDF).</t>
+          <t>Sports chiropractor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Horrigan, Joseph, DC</t>
+          <t>Jamie Shortz</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>scuhs.edu</t>
+          <t>pacificperformancechiro.com</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -7417,19 +7806,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Faculty bio page; no CV.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moreau, William (Bill), DC, DACBSP</t>
+          <t>Joe Jaime</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>neurosportspineandconcussion.com</t>
+          <t>onthegosportschiro.com</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -7444,19 +7833,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Team page with a CV summary and drop-downs; a Curriculum Vitae page with highlights and a "Download Full Curriculum Vitae (PDF)" button; instructor and speaker bios elsewhere.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P2 Sports Care</t>
+          <t>Joel Bienenfeld</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>p2sportscare.com</t>
+          <t>drjoelchiropractic.com</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -7471,19 +7860,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Team page with a full bio for each doctor; no separate CV.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sorrentino, Anne, DC</t>
+          <t>Michael T. Fanning DC, DACBSP, RMSK, CSCS, *D</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>drannesorrentino.com</t>
+          <t>scuhs.edu</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -7498,34 +7887,115 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Short bio with credentials after the name; no CV.</t>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Young, Tom, DC</t>
+          <t>Moreau, William</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>countryside-chiropractic.com</t>
+          <t>neurosportspineandconcussion.com</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sports chiropractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Moreau, William</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>static1.squarespace.com</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sports chiropractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Moreau, William</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>static1.squarespace.com</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>open the CV</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sports chiropractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Robinson Le</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tuneupsmorganhill.com</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
           <t>open the page</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Short bio with credentials after the name; no CV.</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CCSP</t>
         </is>
       </c>
     </row>
@@ -7551,346 +8021,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="47" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Doctor</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Hosted on</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Every saved copy</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Alexis Griffith</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>impowersportsperformance.com</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bart Green</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>nuhs.edu</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Christian Brown</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>dhaj7-cepo.com</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Jamie Shortz</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>pacificperformancechiro.com</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Joe Jaime</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>onthegosportschiro.com</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>open the CV</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Joel Bienenfeld</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>drjoelchiropractic.com</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Michael T. Fanning DC, DACBSP, RMSK, CSCS, *D</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>scuhs.edu</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Moreau, William</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>static1.squarespace.com</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>open the CV</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Sports chiropractor</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Moreau, William</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>static1.squarespace.com</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>open the CV</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Sports chiropractor</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Robinson Le</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>tuneupsmorganhill.com</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>open the page</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>CCSP</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Wayback links open the latest saved page instead of the search page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/cv.xlsx
+++ b/downloads/cv.xlsx
@@ -981,7 +981,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1882,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3730,7 +3730,7 @@
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3906,7 @@
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3950,7 +3950,7 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -3994,7 +3994,7 @@
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4192,7 @@
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4522,7 +4522,7 @@
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -4937,7 +4937,7 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5310,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5398,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5442,7 +5442,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5508,7 +5508,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5552,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5662,7 +5662,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5706,7 +5706,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5728,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5772,7 +5772,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5838,7 +5838,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -5992,7 +5992,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6058,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6102,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6212,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6234,7 +6234,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6278,7 +6278,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6300,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6344,7 +6344,7 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6388,7 +6388,7 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6410,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6454,7 +6454,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6700,7 +6700,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6722,7 +6722,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6788,7 +6788,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6832,7 +6832,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6854,7 +6854,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6898,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6920,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6942,7 +6942,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -6986,7 +6986,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7096,7 +7096,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7162,7 +7162,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7184,7 +7184,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7206,7 +7206,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7228,7 +7228,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7294,7 +7294,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7316,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7382,7 +7382,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7404,7 +7404,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7448,7 +7448,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7470,7 +7470,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7492,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7514,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
     </row>
@@ -7617,7 +7617,7 @@
     <col width="47" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -7666,7 +7666,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -7882,7 +7882,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -7936,7 +7936,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -7963,7 +7963,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Wayback</t>
+          <t>latest saved copy</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">

</xml_diff>